<commit_message>
new changes for task
</commit_message>
<xml_diff>
--- a/cypress/downloads/Client_Summary.xlsx
+++ b/cypress/downloads/Client_Summary.xlsx
@@ -100,10 +100,10 @@
     <x:t>13</x:t>
   </x:si>
   <x:si>
-    <x:t>189</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27/09/23</x:t>
+    <x:t>199</x:t>
+  </x:si>
+  <x:si>
+    <x:t>05/10/23</x:t>
   </x:si>
   <x:si>
     <x:t>Owner nabeel</x:t>

</xml_diff>